<commit_message>
feat: permitir edicao de R$/Ton para frete Hidracor CIF e atualizar bases
</commit_message>
<xml_diff>
--- a/public/Cadastro Clientes Cerbras.xlsx
+++ b/public/Cadastro Clientes Cerbras.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\Nova pasta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F457B1-C3FE-4BAD-9D56-0C806F9BC318}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3F6911-6454-4D60-AA26-E2FBEA4B1EB8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4793" uniqueCount="2622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4805" uniqueCount="2629">
   <si>
     <t>Cliente</t>
   </si>
@@ -7897,6 +7897,27 @@
   </si>
   <si>
     <t>T T OLIVEIRA LTDA - Filial</t>
+  </si>
+  <si>
+    <t>CASA DO CRIADOR E MATERIAIS PARA CONSTRUCAO LTDA</t>
+  </si>
+  <si>
+    <t>20.026.370/0001-05</t>
+  </si>
+  <si>
+    <t>Governador Luiz Rocha</t>
+  </si>
+  <si>
+    <t>IMOBILIARIA SÃO LOURENCO LTDA</t>
+  </si>
+  <si>
+    <t>63.494.470/0001-79</t>
+  </si>
+  <si>
+    <t>CRA ENGENHARIA LTDA</t>
+  </si>
+  <si>
+    <t>63.333.879/0001-03</t>
   </si>
 </sst>
 </file>
@@ -7952,8 +7973,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A3:E1196">
-  <autoFilter ref="A3:E1196" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A3:E1199">
+  <autoFilter ref="A3:E1199" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:E1196">
     <sortCondition ref="A3:A1196"/>
   </sortState>
@@ -8265,7 +8286,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A3:E1196"/>
+  <dimension ref="A3:E1199"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="69.28515625" bestFit="1" customWidth="1"/>
@@ -25042,6 +25063,48 @@
         <v>3</v>
       </c>
     </row>
+    <row r="1197" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1197" t="s">
+        <v>2622</v>
+      </c>
+      <c r="B1197" t="s">
+        <v>2623</v>
+      </c>
+      <c r="C1197" t="s">
+        <v>2624</v>
+      </c>
+      <c r="D1197" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1198" t="s">
+        <v>2625</v>
+      </c>
+      <c r="B1198" t="s">
+        <v>2626</v>
+      </c>
+      <c r="C1198" t="s">
+        <v>2468</v>
+      </c>
+      <c r="D1198" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1199" t="s">
+        <v>2627</v>
+      </c>
+      <c r="B1199" t="s">
+        <v>2628</v>
+      </c>
+      <c r="C1199" t="s">
+        <v>836</v>
+      </c>
+      <c r="D1199" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Ajuste na normalizacao de formatos para importacao de tabelas Cerbras
</commit_message>
<xml_diff>
--- a/public/Cadastro Clientes Cerbras.xlsx
+++ b/public/Cadastro Clientes Cerbras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3F6911-6454-4D60-AA26-E2FBEA4B1EB8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931856F4-F045-45BA-A530-C772787D2640}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4805" uniqueCount="2629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4806" uniqueCount="2629">
   <si>
     <t>Cliente</t>
   </si>
@@ -7975,9 +7975,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A3:E1199">
   <autoFilter ref="A3:E1199" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:E1196">
-    <sortCondition ref="A3:A1196"/>
-  </sortState>
   <tableColumns count="5">
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Cliente"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="CPF_CNPJ_"/>
@@ -24404,6 +24401,9 @@
       <c r="D1149" t="s">
         <v>3</v>
       </c>
+      <c r="E1149" t="s">
+        <v>2619</v>
+      </c>
     </row>
     <row r="1150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1150" t="s">

</xml_diff>

<commit_message>
feat: filter out quotations from detailed and summary financial reports
</commit_message>
<xml_diff>
--- a/public/Cadastro Clientes Cerbras.xlsx
+++ b/public/Cadastro Clientes Cerbras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931856F4-F045-45BA-A530-C772787D2640}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB1458E-CB09-424C-8C1E-EC0A9392F471}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4806" uniqueCount="2629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4807" uniqueCount="2629">
   <si>
     <t>Cliente</t>
   </si>
@@ -11643,7 +11643,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>2193</v>
       </c>
@@ -11657,7 +11657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>1058</v>
       </c>
@@ -11671,7 +11671,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>39</v>
       </c>
@@ -11685,7 +11685,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>751</v>
       </c>
@@ -11699,7 +11699,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>1694</v>
       </c>
@@ -11713,7 +11713,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>1574</v>
       </c>
@@ -11727,7 +11727,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>1151</v>
       </c>
@@ -11741,7 +11741,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>753</v>
       </c>
@@ -11755,7 +11755,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>1359</v>
       </c>
@@ -11769,7 +11769,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>1136</v>
       </c>
@@ -11783,7 +11783,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>2064</v>
       </c>
@@ -11797,7 +11797,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>559</v>
       </c>
@@ -11811,7 +11811,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>290</v>
       </c>
@@ -11825,7 +11825,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>414</v>
       </c>
@@ -11839,7 +11839,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>1792</v>
       </c>
@@ -11852,8 +11852,11 @@
       <c r="D255" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E255" t="s">
+        <v>2619</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>1397</v>
       </c>

</xml_diff>

<commit_message>
fix: resolve white screen when editing closed load and add history filters
</commit_message>
<xml_diff>
--- a/public/Cadastro Clientes Cerbras.xlsx
+++ b/public/Cadastro Clientes Cerbras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB1458E-CB09-424C-8C1E-EC0A9392F471}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E88A427C-98DF-4B58-8610-A49ED53F4E18}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4807" uniqueCount="2629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4808" uniqueCount="2629">
   <si>
     <t>Cliente</t>
   </si>
@@ -17255,7 +17255,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="641" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="641" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A641" t="s">
         <v>659</v>
       </c>
@@ -17269,7 +17269,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="642" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="642" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A642" t="s">
         <v>2005</v>
       </c>
@@ -17283,7 +17283,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="643" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="643" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A643" t="s">
         <v>49</v>
       </c>
@@ -17297,7 +17297,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="644" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="644" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A644" t="s">
         <v>1227</v>
       </c>
@@ -17311,7 +17311,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="645" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="645" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A645" t="s">
         <v>2332</v>
       </c>
@@ -17324,8 +17324,11 @@
       <c r="D645" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="646" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E645" t="s">
+        <v>2619</v>
+      </c>
+    </row>
+    <row r="646" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A646" t="s">
         <v>1284</v>
       </c>
@@ -17339,7 +17342,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="647" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="647" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A647" t="s">
         <v>208</v>
       </c>
@@ -17353,7 +17356,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="648" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="648" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A648" t="s">
         <v>64</v>
       </c>
@@ -17367,7 +17370,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="649" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="649" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A649" t="s">
         <v>1933</v>
       </c>
@@ -17381,7 +17384,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="650" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="650" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A650" t="s">
         <v>1497</v>
       </c>
@@ -17395,7 +17398,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="651" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="651" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A651" t="s">
         <v>1499</v>
       </c>
@@ -17409,7 +17412,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="652" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="652" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A652" t="s">
         <v>2444</v>
       </c>
@@ -17423,7 +17426,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="653" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="653" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A653" t="s">
         <v>1083</v>
       </c>
@@ -17437,7 +17440,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="654" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="654" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A654" t="s">
         <v>885</v>
       </c>
@@ -17451,7 +17454,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="655" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="655" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A655" t="s">
         <v>2118</v>
       </c>
@@ -17465,7 +17468,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="656" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="656" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A656" t="s">
         <v>1501</v>
       </c>

</xml_diff>

<commit_message>
chore: atualiza planilhas de fretes e cadastros de clientes
</commit_message>
<xml_diff>
--- a/public/Cadastro Clientes Cerbras.xlsx
+++ b/public/Cadastro Clientes Cerbras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\MIDAS RENT A CAR\midas-log\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E88A427C-98DF-4B58-8610-A49ED53F4E18}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609F852E-B652-418A-974C-1CC98EC2AE19}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4808" uniqueCount="2629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4809" uniqueCount="2629">
   <si>
     <t>Cliente</t>
   </si>
@@ -21747,7 +21747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="961" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="961" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A961" t="s">
         <v>2374</v>
       </c>
@@ -21761,7 +21761,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="962" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="962" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A962" t="s">
         <v>256</v>
       </c>
@@ -21775,7 +21775,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="963" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="963" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A963" t="s">
         <v>318</v>
       </c>
@@ -21789,7 +21789,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="964" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="964" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A964" t="s">
         <v>1373</v>
       </c>
@@ -21803,7 +21803,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="965" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="965" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A965" t="s">
         <v>1651</v>
       </c>
@@ -21817,7 +21817,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="966" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="966" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A966" t="s">
         <v>855</v>
       </c>
@@ -21830,8 +21830,11 @@
       <c r="D966" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="967" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E966" t="s">
+        <v>2619</v>
+      </c>
+    </row>
+    <row r="967" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A967" t="s">
         <v>2505</v>
       </c>
@@ -21845,7 +21848,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="968" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="968" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A968" t="s">
         <v>986</v>
       </c>
@@ -21859,7 +21862,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="969" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="969" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A969" t="s">
         <v>2377</v>
       </c>
@@ -21873,7 +21876,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="970" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="970" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A970" t="s">
         <v>2606</v>
       </c>
@@ -21887,7 +21890,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="971" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="971" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A971" t="s">
         <v>675</v>
       </c>
@@ -21901,7 +21904,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="972" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="972" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A972" t="s">
         <v>809</v>
       </c>
@@ -21915,7 +21918,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="973" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="973" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A973" t="s">
         <v>399</v>
       </c>
@@ -21929,7 +21932,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="974" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="974" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A974" t="s">
         <v>2238</v>
       </c>
@@ -21943,7 +21946,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="975" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="975" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A975" t="s">
         <v>2238</v>
       </c>
@@ -21957,7 +21960,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="976" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="976" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A976" t="s">
         <v>638</v>
       </c>

</xml_diff>